<commit_message>
Update Mente Brilhante badge threshold
</commit_message>
<xml_diff>
--- a/Tratamento - base 2026.xlsx
+++ b/Tratamento - base 2026.xlsx
@@ -1144,11 +1144,7 @@
       </c>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AL5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2003,11 +1999,7 @@
         </is>
       </c>
       <c r="AJ12" t="inlineStr"/>
-      <c r="AK12" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AK12" t="inlineStr"/>
       <c r="AL12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -2740,11 +2732,7 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="AL18" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AL18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2987,11 +2975,7 @@
         </is>
       </c>
       <c r="AJ20" t="inlineStr"/>
-      <c r="AK20" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -3476,11 +3460,7 @@
       </c>
       <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr"/>
-      <c r="AL24" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AL24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3600,11 +3580,7 @@
       </c>
       <c r="AJ25" t="inlineStr"/>
       <c r="AK25" t="inlineStr"/>
-      <c r="AL25" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AL25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3844,11 +3820,7 @@
       </c>
       <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr"/>
-      <c r="AL27" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AL27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4948,11 +4920,7 @@
       </c>
       <c r="AJ36" t="inlineStr"/>
       <c r="AK36" t="inlineStr"/>
-      <c r="AL36" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AL36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5552,11 +5520,7 @@
       </c>
       <c r="AJ41" t="inlineStr"/>
       <c r="AK41" t="inlineStr"/>
-      <c r="AL41" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AL41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6036,11 +6000,7 @@
       </c>
       <c r="AJ45" t="inlineStr"/>
       <c r="AK45" t="inlineStr"/>
-      <c r="AL45" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AL45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6160,11 +6120,7 @@
       </c>
       <c r="AJ46" t="inlineStr"/>
       <c r="AK46" t="inlineStr"/>
-      <c r="AL46" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
+      <c r="AL46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">

</xml_diff>